<commit_message>
Implement SQLite queue backend
</commit_message>
<xml_diff>
--- a/share/config/orqflow_v0_1/Input/Input01.xlsx
+++ b/share/config/orqflow_v0_1/Input/Input01.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\share\config\orqflow_v0_1\Input\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Document\PyProject\Playwright\OrqFlow_V0.1\share\config\orqflow_v0_1\Input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D163653-CE4C-4B30-89BB-AB7C2845682F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB3C0195-BADB-41B1-805C-5B8A9FB27C74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2085" windowWidth="28800" windowHeight="13395" xr2:uid="{2CE5C760-F4B0-4544-B529-E47EF909E11F}"/>
+    <workbookView xWindow="5580" yWindow="2400" windowWidth="28800" windowHeight="13395" xr2:uid="{2CE5C760-F4B0-4544-B529-E47EF909E11F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,27 +34,93 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="7">
-  <si>
-    <t>TransID</t>
-  </si>
-  <si>
-    <t>InputDetails</t>
-  </si>
-  <si>
-    <t>OutputDetails</t>
-  </si>
-  <si>
-    <t>Status</t>
-  </si>
-  <si>
-    <t>Test Input1</t>
-  </si>
-  <si>
-    <t>Test Input2</t>
-  </si>
-  <si>
-    <t>Queue Created</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="29">
+  <si>
+    <t>Processor</t>
+  </si>
+  <si>
+    <t>Process</t>
+  </si>
+  <si>
+    <t>Case_Number</t>
+  </si>
+  <si>
+    <t>Transaction_ID</t>
+  </si>
+  <si>
+    <t>Case_Status</t>
+  </si>
+  <si>
+    <t>Chargeback_Date</t>
+  </si>
+  <si>
+    <t>Case_Json</t>
+  </si>
+  <si>
+    <t>Transaction_Amount</t>
+  </si>
+  <si>
+    <t>Mid_Alias</t>
+  </si>
+  <si>
+    <t>MID_Number</t>
+  </si>
+  <si>
+    <t>Case_ID</t>
+  </si>
+  <si>
+    <t>Chargeback_Amount</t>
+  </si>
+  <si>
+    <t>Transaction_Date</t>
+  </si>
+  <si>
+    <t>Deadline_Date</t>
+  </si>
+  <si>
+    <t>Card_First_Six</t>
+  </si>
+  <si>
+    <t>Card_Last_Four</t>
+  </si>
+  <si>
+    <t>Card_Type</t>
+  </si>
+  <si>
+    <t>Institution</t>
+  </si>
+  <si>
+    <t>BUnit</t>
+  </si>
+  <si>
+    <t>Fiserv</t>
+  </si>
+  <si>
+    <t>Test000001</t>
+  </si>
+  <si>
+    <t>Test000002</t>
+  </si>
+  <si>
+    <t>{}</t>
+  </si>
+  <si>
+    <t>Dummy_Alias</t>
+  </si>
+  <si>
+    <t>000000</t>
+  </si>
+  <si>
+    <t>0000</t>
+  </si>
+  <si>
+    <t>Visa</t>
+  </si>
+  <si>
+    <t>AT&amp;T</t>
+  </si>
+  <si>
+    <t>Entertainment</t>
   </si>
 </sst>
 </file>
@@ -90,8 +156,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -110,13 +178,28 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F1A7D28B-8B98-4259-91FA-5A4F733D83B9}" name="Table1" displayName="Table1" ref="A1:D3" totalsRowShown="0">
-  <autoFilter ref="A1:D3" xr:uid="{F1A7D28B-8B98-4259-91FA-5A4F733D83B9}"/>
-  <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{B7E4FCE3-E576-47CD-A5AE-241248E6BB57}" name="TransID"/>
-    <tableColumn id="2" xr3:uid="{A691E098-F03C-4D6B-9337-BC015C5979A0}" name="InputDetails"/>
-    <tableColumn id="3" xr3:uid="{1D5211D7-7382-41C8-B4F0-848870EC61D2}" name="OutputDetails"/>
-    <tableColumn id="4" xr3:uid="{97B89EA1-94DD-4A2F-860F-FB4E7282B2FA}" name="Status"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F1A7D28B-8B98-4259-91FA-5A4F733D83B9}" name="Table1" displayName="Table1" ref="A1:S3" totalsRowShown="0">
+  <autoFilter ref="A1:S3" xr:uid="{F1A7D28B-8B98-4259-91FA-5A4F733D83B9}"/>
+  <tableColumns count="19">
+    <tableColumn id="2" xr3:uid="{A691E098-F03C-4D6B-9337-BC015C5979A0}" name="Processor"/>
+    <tableColumn id="3" xr3:uid="{1D5211D7-7382-41C8-B4F0-848870EC61D2}" name="Process"/>
+    <tableColumn id="4" xr3:uid="{97B89EA1-94DD-4A2F-860F-FB4E7282B2FA}" name="Case_Number"/>
+    <tableColumn id="5" xr3:uid="{41C1FA18-05C0-4309-8054-CDEC66D47726}" name="Transaction_ID"/>
+    <tableColumn id="6" xr3:uid="{A085BF32-FEC0-4956-9475-912777094851}" name="Case_Status"/>
+    <tableColumn id="7" xr3:uid="{115B0AAA-0C77-4B59-8197-C5EB0B04F410}" name="Chargeback_Date"/>
+    <tableColumn id="8" xr3:uid="{F1D7F57B-3DC2-41B8-8B29-89C4B05BDC1D}" name="Case_Json"/>
+    <tableColumn id="9" xr3:uid="{420006C7-EF1A-4A12-92FB-9EEF625DAA38}" name="Transaction_Amount"/>
+    <tableColumn id="10" xr3:uid="{51C6F895-B303-4195-90FA-E6DE5E2ACBEF}" name="Mid_Alias"/>
+    <tableColumn id="11" xr3:uid="{326D4106-534F-47AB-8C34-3BE23D5820C6}" name="MID_Number"/>
+    <tableColumn id="12" xr3:uid="{1ED5190C-02D1-4F73-B284-38718DF27872}" name="Case_ID"/>
+    <tableColumn id="13" xr3:uid="{33E91E2D-F0B0-47C2-8491-DAF3BD7BFC69}" name="Chargeback_Amount"/>
+    <tableColumn id="14" xr3:uid="{7AA00EA8-986D-4260-AC08-F6323601748B}" name="Transaction_Date"/>
+    <tableColumn id="15" xr3:uid="{C6F924BE-DA09-4A56-8071-822FAF69CFD2}" name="Deadline_Date"/>
+    <tableColumn id="16" xr3:uid="{30DBF390-4493-4CDF-B852-855D127662FE}" name="Card_First_Six"/>
+    <tableColumn id="17" xr3:uid="{F81C7806-58C3-4E07-B82D-67C51EAADA66}" name="Card_Last_Four"/>
+    <tableColumn id="18" xr3:uid="{7A31265C-308E-4500-A25E-80F430BB1DD5}" name="Card_Type"/>
+    <tableColumn id="22" xr3:uid="{F0F14A7E-D0A7-4975-B829-D491DB231BF4}" name="Institution"/>
+    <tableColumn id="23" xr3:uid="{FDA266D8-CF48-4C88-9387-DBA6609BE284}" name="BUnit"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -419,15 +502,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7E20557-FA5E-4231-BE97-AFC5317631CD}">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:S3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.7109375" customWidth="1"/>
-    <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="3" width="15.5703125" customWidth="1"/>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="15.5703125" customWidth="1"/>
+    <col min="3" max="3" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="14" width="10.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -440,27 +525,156 @@
       <c r="D1" t="s">
         <v>3</v>
       </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" t="s">
+        <v>18</v>
+      </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D2" t="s">
-        <v>6</v>
+    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2">
+        <v>11</v>
+      </c>
+      <c r="C2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F2" s="1">
+        <v>46023</v>
+      </c>
+      <c r="G2" t="s">
+        <v>22</v>
+      </c>
+      <c r="H2">
+        <v>1000.01</v>
+      </c>
+      <c r="I2" t="s">
+        <v>23</v>
+      </c>
+      <c r="J2">
+        <v>100001</v>
+      </c>
+      <c r="K2">
+        <v>1000001</v>
+      </c>
+      <c r="L2">
+        <v>100.01</v>
+      </c>
+      <c r="M2" s="1">
+        <v>46037</v>
+      </c>
+      <c r="N2" s="1">
+        <v>46047</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="P2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>26</v>
+      </c>
+      <c r="R2" t="s">
+        <v>27</v>
+      </c>
+      <c r="S2" t="s">
+        <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D3" t="s">
-        <v>6</v>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3">
+        <v>11</v>
+      </c>
+      <c r="C3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F3" s="1">
+        <v>46023</v>
+      </c>
+      <c r="G3" t="s">
+        <v>22</v>
+      </c>
+      <c r="H3">
+        <v>1000.01</v>
+      </c>
+      <c r="I3" t="s">
+        <v>23</v>
+      </c>
+      <c r="J3">
+        <v>100001</v>
+      </c>
+      <c r="K3">
+        <v>1000001</v>
+      </c>
+      <c r="L3">
+        <v>100.01</v>
+      </c>
+      <c r="M3" s="1">
+        <v>46037</v>
+      </c>
+      <c r="N3" s="1">
+        <v>46047</v>
+      </c>
+      <c r="O3" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="P3" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>26</v>
+      </c>
+      <c r="R3" t="s">
+        <v>27</v>
+      </c>
+      <c r="S3" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Improve master queue input handling
</commit_message>
<xml_diff>
--- a/share/config/orqflow_v0_1/Input/Input01.xlsx
+++ b/share/config/orqflow_v0_1/Input/Input01.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Document\PyProject\Playwright\OrqFlow_V0.1\share\config\orqflow_v0_1\Input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB3C0195-BADB-41B1-805C-5B8A9FB27C74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08C47C03-75E5-4014-8C75-9C06169DA901}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5580" yWindow="2400" windowWidth="28800" windowHeight="13395" xr2:uid="{2CE5C760-F4B0-4544-B529-E47EF909E11F}"/>
+    <workbookView xWindow="0" yWindow="1020" windowWidth="28800" windowHeight="13395" xr2:uid="{2CE5C760-F4B0-4544-B529-E47EF909E11F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,12 +34,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="28">
   <si>
     <t>Processor</t>
-  </si>
-  <si>
-    <t>Process</t>
   </si>
   <si>
     <t>Case_Number</t>
@@ -178,11 +175,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F1A7D28B-8B98-4259-91FA-5A4F733D83B9}" name="Table1" displayName="Table1" ref="A1:S3" totalsRowShown="0">
-  <autoFilter ref="A1:S3" xr:uid="{F1A7D28B-8B98-4259-91FA-5A4F733D83B9}"/>
-  <tableColumns count="19">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F1A7D28B-8B98-4259-91FA-5A4F733D83B9}" name="Table1" displayName="Table1" ref="A1:R3" totalsRowShown="0">
+  <autoFilter ref="A1:R3" xr:uid="{F1A7D28B-8B98-4259-91FA-5A4F733D83B9}"/>
+  <tableColumns count="18">
     <tableColumn id="2" xr3:uid="{A691E098-F03C-4D6B-9337-BC015C5979A0}" name="Processor"/>
-    <tableColumn id="3" xr3:uid="{1D5211D7-7382-41C8-B4F0-848870EC61D2}" name="Process"/>
     <tableColumn id="4" xr3:uid="{97B89EA1-94DD-4A2F-860F-FB4E7282B2FA}" name="Case_Number"/>
     <tableColumn id="5" xr3:uid="{41C1FA18-05C0-4309-8054-CDEC66D47726}" name="Transaction_ID"/>
     <tableColumn id="6" xr3:uid="{A085BF32-FEC0-4956-9475-912777094851}" name="Case_Status"/>
@@ -502,17 +498,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7E20557-FA5E-4231-BE97-AFC5317631CD}">
-  <dimension ref="A1:S3"/>
+  <dimension ref="A1:R3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="15.5703125" customWidth="1"/>
-    <col min="3" max="3" width="15.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="14" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="12" max="13" width="10.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -567,51 +562,48 @@
       <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="B2" t="s">
         <v>19</v>
       </c>
-      <c r="B2">
-        <v>11</v>
-      </c>
-      <c r="C2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F2" s="1">
+      <c r="E2" s="1">
         <v>46023</v>
       </c>
-      <c r="G2" t="s">
+      <c r="F2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G2">
+        <v>1000.01</v>
+      </c>
+      <c r="H2" t="s">
         <v>22</v>
       </c>
-      <c r="H2">
-        <v>1000.01</v>
-      </c>
-      <c r="I2" t="s">
+      <c r="I2">
+        <v>100001</v>
+      </c>
+      <c r="J2">
+        <v>1000001</v>
+      </c>
+      <c r="K2">
+        <v>100.01</v>
+      </c>
+      <c r="L2" s="1">
+        <v>46037</v>
+      </c>
+      <c r="M2" s="1">
+        <v>46047</v>
+      </c>
+      <c r="N2" s="2" t="s">
         <v>23</v>
-      </c>
-      <c r="J2">
-        <v>100001</v>
-      </c>
-      <c r="K2">
-        <v>1000001</v>
-      </c>
-      <c r="L2">
-        <v>100.01</v>
-      </c>
-      <c r="M2" s="1">
-        <v>46037</v>
-      </c>
-      <c r="N2" s="1">
-        <v>46047</v>
       </c>
       <c r="O2" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="P2" s="2" t="s">
+      <c r="P2" t="s">
         <v>25</v>
       </c>
       <c r="Q2" t="s">
@@ -620,51 +612,48 @@
       <c r="R2" t="s">
         <v>27</v>
       </c>
-      <c r="S2" t="s">
-        <v>28</v>
-      </c>
     </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>19</v>
-      </c>
-      <c r="B3">
-        <v>11</v>
-      </c>
-      <c r="C3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E3" s="1">
+        <v>46023</v>
+      </c>
+      <c r="F3" t="s">
         <v>21</v>
       </c>
-      <c r="F3" s="1">
-        <v>46023</v>
-      </c>
-      <c r="G3" t="s">
+      <c r="G3">
+        <v>1000.01</v>
+      </c>
+      <c r="H3" t="s">
         <v>22</v>
       </c>
-      <c r="H3">
-        <v>1000.01</v>
-      </c>
-      <c r="I3" t="s">
+      <c r="I3">
+        <v>100001</v>
+      </c>
+      <c r="J3">
+        <v>1000001</v>
+      </c>
+      <c r="K3">
+        <v>100.01</v>
+      </c>
+      <c r="L3" s="1">
+        <v>46037</v>
+      </c>
+      <c r="M3" s="1">
+        <v>46047</v>
+      </c>
+      <c r="N3" s="2" t="s">
         <v>23</v>
-      </c>
-      <c r="J3">
-        <v>100001</v>
-      </c>
-      <c r="K3">
-        <v>1000001</v>
-      </c>
-      <c r="L3">
-        <v>100.01</v>
-      </c>
-      <c r="M3" s="1">
-        <v>46037</v>
-      </c>
-      <c r="N3" s="1">
-        <v>46047</v>
       </c>
       <c r="O3" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="P3" s="2" t="s">
+      <c r="P3" t="s">
         <v>25</v>
       </c>
       <c r="Q3" t="s">
@@ -672,9 +661,6 @@
       </c>
       <c r="R3" t="s">
         <v>27</v>
-      </c>
-      <c r="S3" t="s">
-        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>